<commit_message>
Add Excel columns and seed resolution for implicit many-to-many relations
Organization<->Country and 5 other implicit M2M relations (no FK column
possible on either side) had no column in the generated Excel templates and
no seed logic at all. Adds a curated free-text ";"-separated column per
relation (organizations.xlsx: countries/industries/working_area_cities,
cities.xlsx: main_industries, subjects.xlsx: industries, industries.xlsx:
related_industries), resolved at seed time via a new seeds_relations.ts that
runs last. Also fixes two pre-existing FK passthrough bugs found in the same
audit: seeds_organizations.ts (city_id/parent_organization_id) and
seeds_jobs.ts (industry_id) were assigning raw CSV strings straight into
UUID columns instead of resolving them by name.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/api/data/excel_templates/cities.xlsx
+++ b/apps/api/data/excel_templates/cities.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z1"/>
+  <dimension ref="A1:AA1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="1" min="1" max="1"/>
@@ -467,6 +467,7 @@
     <col width="18" customWidth="1" style="4" min="24" max="24"/>
     <col width="18" customWidth="1" style="4" min="25" max="25"/>
     <col width="18" customWidth="1" style="1" min="26" max="26"/>
+    <col width="19" customWidth="1" style="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -598,6 +599,11 @@
       <c r="Z1" s="6" t="inlineStr">
         <is>
           <t>metadata</t>
+        </is>
+      </c>
+      <c r="AA1" s="6" t="inlineStr">
+        <is>
+          <t>main_industries</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Renseigne state_province sur les 3 lignes Alexandria
cities.csv contenait trois "Alexandria" (EG/RO/US) sans state_province :
rien ne permettait de trancher, donc les 4 organisations situées à
Alexandria, Virginia tombaient à null.

Rempli dans cities.xlsx (source de vérité, le CSV en étant régénéré par
excel_to_csv.py) selon la convention du fichier - division administrative
de premier niveau en toutes lettres, comme Massachusetts/England/Ontario :
CIT-000056 (EG) -> Alexandria, CIT-000057 (RO) -> Teleorman,
CIT-000058 (US) -> Virginia.

"Alexandria, Virginia" résout désormais vers CIT-000058 ; "Alexandria"
seul reste null, toujours ambigu. Les avertissements city_name passent de
84 à 80.

Vérifié : 9 validations de données, protection de feuille et lockStructure
intactes après enregistrement openpyxl ; aller-retour xlsx -> csv identique
au octet près sur les 10 modèles ; diff CSV limité à ces 3 cellules ;
17/17 tests du moteur.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/api/data/excel_templates/cities.xlsx
+++ b/apps/api/data/excel_templates/cities.xlsx
@@ -6068,6 +6068,11 @@
           <t>EG</t>
         </is>
       </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Alexandria</t>
+        </is>
+      </c>
       <c r="F57" t="inlineStr">
         <is>
           <t>5.2 million (Foreign Born: 300,000)</t>
@@ -6167,6 +6172,11 @@
           <t>RO</t>
         </is>
       </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Teleorman</t>
+        </is>
+      </c>
       <c r="F58" t="inlineStr">
         <is>
           <t>300,000 (Foreign Born: 8,000)</t>
@@ -6264,6 +6274,11 @@
       <c r="C59" t="inlineStr">
         <is>
           <t>US</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Virginia</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">

</xml_diff>